<commit_message>
feat: integrate official certificate template with dynamic conference & student text + bundled fonts
</commit_message>
<xml_diff>
--- a/data/accounting.xlsx
+++ b/data/accounting.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,6 +493,20 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>طارق ابراهيم مصطفى</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ريم خالد السيد</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>